<commit_message>
Update NBA features + predictions: 2026-09-29 14:09
</commit_message>
<xml_diff>
--- a/nba-backend/data_delivery/nba_feature_workbook_20260929.xlsx
+++ b/nba-backend/data_delivery/nba_feature_workbook_20260929.xlsx
@@ -9356,7 +9356,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>25.1162</v>
+        <v>91.0172</v>
       </c>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
@@ -9365,11 +9365,11 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>ewm_def_rating_diff</t>
+          <t>ewm_off_rating_diff</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>6.5066</v>
+        <v>1.7024</v>
       </c>
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="n"/>
@@ -9378,11 +9378,11 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ewm_off_rating_diff</t>
+          <t>ewm_def_rating_diff</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>5.7203</v>
+        <v>1.6724</v>
       </c>
       <c r="C19" s="2" t="n"/>
       <c r="D19" s="2" t="n"/>
@@ -9395,7 +9395,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>4.0509</v>
+        <v>1.598</v>
       </c>
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n"/>
@@ -9404,11 +9404,11 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>elo_away</t>
+          <t>ewm_rebound_margin_diff</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>1.5027</v>
+        <v>0.724</v>
       </c>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
@@ -9417,11 +9417,11 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>elo_home</t>
+          <t>rest_days_diff</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>1.4994</v>
+        <v>0.4922</v>
       </c>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n"/>
@@ -9430,11 +9430,11 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ewm_off_rating_away</t>
+          <t>ewm_turnover_margin_diff</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>1.4675</v>
+        <v>0.277</v>
       </c>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n"/>
@@ -9443,11 +9443,11 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ewm_rebound_margin_diff</t>
+          <t>back_to_back_diff</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>1.3425</v>
+        <v>0.1106</v>
       </c>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
@@ -9456,11 +9456,11 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_away</t>
+          <t>elo_home</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1.2721</v>
+        <v>0.08110000000000001</v>
       </c>
       <c r="C25" s="2" t="n"/>
       <c r="D25" s="2" t="n"/>
@@ -9469,11 +9469,11 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>win_pct_diff</t>
+          <t>pl_ts_c_away</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>1.2512</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="n"/>
@@ -9592,7 +9592,7 @@
         <v>100</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>25.1162</v>
+        <v>91.0172</v>
       </c>
     </row>
     <row r="3">
@@ -9635,7 +9635,7 @@
         <v>100</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>1.2512</v>
+        <v>0.0413</v>
       </c>
     </row>
     <row r="4">
@@ -9678,7 +9678,7 @@
         <v>100</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>1.0549</v>
+        <v>0.4922</v>
       </c>
     </row>
     <row r="5">
@@ -9721,7 +9721,7 @@
         <v>100</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.7059</v>
+        <v>0.1106</v>
       </c>
     </row>
     <row r="6">
@@ -9764,7 +9764,7 @@
         <v>100</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>4.0509</v>
+        <v>1.598</v>
       </c>
     </row>
     <row r="7">
@@ -9807,7 +9807,7 @@
         <v>100</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>5.7203</v>
+        <v>1.7024</v>
       </c>
     </row>
     <row r="8">
@@ -9850,7 +9850,7 @@
         <v>100</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>6.5066</v>
+        <v>1.6724</v>
       </c>
     </row>
     <row r="9">
@@ -9893,7 +9893,7 @@
         <v>100</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0.6393</v>
+        <v>0.0303</v>
       </c>
     </row>
     <row r="10">
@@ -9936,7 +9936,7 @@
         <v>100</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.7682</v>
+        <v>0.0346</v>
       </c>
     </row>
     <row r="11">
@@ -9979,7 +9979,7 @@
         <v>100</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.9045</v>
+        <v>0.277</v>
       </c>
     </row>
     <row r="12">
@@ -10022,7 +10022,7 @@
         <v>100</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>1.3425</v>
+        <v>0.724</v>
       </c>
     </row>
     <row r="13">
@@ -10065,7 +10065,7 @@
         <v>100</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>1.0841</v>
+        <v>0.047</v>
       </c>
     </row>
     <row r="14">
@@ -10108,7 +10108,7 @@
         <v>100</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.7</v>
+        <v>0.0023</v>
       </c>
     </row>
     <row r="15">
@@ -10151,7 +10151,7 @@
         <v>100</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>1.4994</v>
+        <v>0.08110000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -10194,7 +10194,7 @@
         <v>100</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>1.5027</v>
+        <v>0.06850000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -10237,7 +10237,7 @@
         <v>100</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0.5279</v>
+        <v>0.0244</v>
       </c>
     </row>
     <row r="18">
@@ -10280,7 +10280,7 @@
         <v>100</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0.8023</v>
+        <v>0.0305</v>
       </c>
     </row>
     <row r="19">
@@ -10323,7 +10323,7 @@
         <v>100</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>1.0957</v>
+        <v>0.0427</v>
       </c>
     </row>
     <row r="20">
@@ -10366,7 +10366,7 @@
         <v>100</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1.4675</v>
+        <v>0.0641</v>
       </c>
     </row>
     <row r="21">
@@ -10409,7 +10409,7 @@
         <v>100</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>1.0067</v>
+        <v>0.0548</v>
       </c>
     </row>
     <row r="22">
@@ -10452,7 +10452,7 @@
         <v>100</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>1.1968</v>
+        <v>0.0497</v>
       </c>
     </row>
     <row r="23">
@@ -10495,7 +10495,7 @@
         <v>100</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>1.106</v>
+        <v>0.0399</v>
       </c>
     </row>
     <row r="24">
@@ -10538,7 +10538,7 @@
         <v>100</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0</v>
+        <v>0.0313</v>
       </c>
     </row>
     <row r="25">
@@ -10581,7 +10581,7 @@
         <v>100</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0.8504</v>
+        <v>0.043</v>
       </c>
     </row>
     <row r="26">
@@ -10624,7 +10624,7 @@
         <v>100</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>0.4797</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -10667,7 +10667,7 @@
         <v>100</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0.8186</v>
+        <v>0.0387</v>
       </c>
     </row>
     <row r="28">
@@ -10710,7 +10710,7 @@
         <v>100</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>1.0342</v>
+        <v>0.0601</v>
       </c>
     </row>
     <row r="29">
@@ -10753,7 +10753,7 @@
         <v>100</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>1.0473</v>
+        <v>0.0432</v>
       </c>
     </row>
     <row r="30">
@@ -10796,7 +10796,7 @@
         <v>100</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0.9177999999999999</v>
+        <v>0.0386</v>
       </c>
     </row>
     <row r="31">
@@ -10839,7 +10839,7 @@
         <v>100</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0.9507</v>
+        <v>0.0463</v>
       </c>
     </row>
     <row r="32">
@@ -10882,7 +10882,7 @@
         <v>100</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0.8407</v>
+        <v>0.0358</v>
       </c>
     </row>
     <row r="33">
@@ -10925,7 +10925,7 @@
         <v>100</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>0.7994</v>
+        <v>0.0409</v>
       </c>
     </row>
     <row r="34">
@@ -10968,7 +10968,7 @@
         <v>100</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0.7863</v>
+        <v>0.0374</v>
       </c>
     </row>
     <row r="35">
@@ -11011,7 +11011,7 @@
         <v>100</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0.9322</v>
+        <v>0.039</v>
       </c>
     </row>
     <row r="36">
@@ -11054,7 +11054,7 @@
         <v>100</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0.7668</v>
+        <v>0.0366</v>
       </c>
     </row>
     <row r="37">
@@ -11097,7 +11097,7 @@
         <v>100</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>0.7635</v>
+        <v>0.027</v>
       </c>
     </row>
     <row r="38">
@@ -11140,7 +11140,7 @@
         <v>100</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0.9029</v>
+        <v>0.0361</v>
       </c>
     </row>
     <row r="39">
@@ -11183,7 +11183,7 @@
         <v>100</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0.7647</v>
+        <v>0.0381</v>
       </c>
     </row>
     <row r="40">
@@ -11226,7 +11226,7 @@
         <v>100</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0.8577</v>
+        <v>0.0372</v>
       </c>
     </row>
     <row r="41">
@@ -11269,7 +11269,7 @@
         <v>100</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>1.0279</v>
+        <v>0.0386</v>
       </c>
     </row>
     <row r="42">
@@ -11312,7 +11312,7 @@
         <v>100</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0.8016</v>
+        <v>0.0331</v>
       </c>
     </row>
     <row r="43">
@@ -11355,7 +11355,7 @@
         <v>100</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0.7861</v>
+        <v>0.0371</v>
       </c>
     </row>
     <row r="44">
@@ -11398,7 +11398,7 @@
         <v>100</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.7359</v>
+        <v>0.0293</v>
       </c>
     </row>
     <row r="45">
@@ -11441,7 +11441,7 @@
         <v>100</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>0.736</v>
+        <v>0.0371</v>
       </c>
     </row>
     <row r="46">
@@ -11484,7 +11484,7 @@
         <v>100</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>0.8363</v>
+        <v>0.0413</v>
       </c>
     </row>
     <row r="47">
@@ -11527,7 +11527,7 @@
         <v>100</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.8976</v>
+        <v>0.0358</v>
       </c>
     </row>
     <row r="48">
@@ -11570,7 +11570,7 @@
         <v>100</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>1.0085</v>
+        <v>0.0364</v>
       </c>
     </row>
     <row r="49">
@@ -11613,7 +11613,7 @@
         <v>100</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>0.7968</v>
+        <v>0.0331</v>
       </c>
     </row>
     <row r="50">
@@ -11656,7 +11656,7 @@
         <v>100</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>0.6751</v>
+        <v>0.0382</v>
       </c>
     </row>
     <row r="51">
@@ -11699,7 +11699,7 @@
         <v>100</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>0.921</v>
+        <v>0.0345</v>
       </c>
     </row>
     <row r="52">
@@ -11742,7 +11742,7 @@
         <v>100</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.7968</v>
+        <v>0.0384</v>
       </c>
     </row>
     <row r="53">
@@ -11785,7 +11785,7 @@
         <v>100</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.9216</v>
+        <v>0.0441</v>
       </c>
     </row>
     <row r="54">
@@ -11828,7 +11828,7 @@
         <v>100</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.9298999999999999</v>
+        <v>0.038</v>
       </c>
     </row>
     <row r="55">
@@ -11914,7 +11914,7 @@
         <v>100</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0.6892</v>
+        <v>0.0387</v>
       </c>
     </row>
     <row r="57">
@@ -11957,7 +11957,7 @@
         <v>100</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.0366</v>
       </c>
     </row>
     <row r="58">
@@ -12000,7 +12000,7 @@
         <v>100</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.843</v>
+        <v>0.0311</v>
       </c>
     </row>
     <row r="59">
@@ -12043,7 +12043,7 @@
         <v>100</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.7106</v>
+        <v>0.0299</v>
       </c>
     </row>
     <row r="60">
@@ -12086,7 +12086,7 @@
         <v>100</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.9939</v>
+        <v>0.0404</v>
       </c>
     </row>
     <row r="61">
@@ -12129,7 +12129,7 @@
         <v>100</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>0.7329</v>
+        <v>0.0217</v>
       </c>
     </row>
     <row r="62">
@@ -12172,7 +12172,7 @@
         <v>100</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>0.8078</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="63">
@@ -12215,7 +12215,7 @@
         <v>100</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>0.8245</v>
+        <v>0.0361</v>
       </c>
     </row>
     <row r="64">
@@ -12258,7 +12258,7 @@
         <v>32.3</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>1.2721</v>
+        <v>0.06900000000000001</v>
       </c>
     </row>
     <row r="65">
@@ -12301,7 +12301,7 @@
         <v>48.4</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>0.6273</v>
+        <v>0.0342</v>
       </c>
     </row>
     <row r="66">
@@ -12344,7 +12344,7 @@
         <v>19.4</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>0.8405</v>
+        <v>0.037</v>
       </c>
     </row>
     <row r="67">
@@ -12387,7 +12387,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>0.8945</v>
+        <v>0.0378</v>
       </c>
     </row>
     <row r="68">
@@ -12430,7 +12430,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0.9424</v>
+        <v>0.0489</v>
       </c>
     </row>
     <row r="69">
@@ -12473,7 +12473,7 @@
         <v>67.7</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>1.0223</v>
+        <v>0.0375</v>
       </c>
     </row>
     <row r="70">
@@ -12516,7 +12516,7 @@
         <v>100</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>0.8672</v>
+        <v>0.0399</v>
       </c>
     </row>
     <row r="71">
@@ -12559,7 +12559,7 @@
         <v>100</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>0.825</v>
+        <v>0.0329</v>
       </c>
     </row>
     <row r="72">
@@ -12602,7 +12602,7 @@
         <v>100</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>0.8192</v>
+        <v>0.0431</v>
       </c>
     </row>
     <row r="73">
@@ -14692,7 +14692,7 @@
         <v>100</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>25.1162</v>
+        <v>91.0172</v>
       </c>
     </row>
     <row r="3">
@@ -14735,7 +14735,7 @@
         <v>100</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>1.2512</v>
+        <v>0.0413</v>
       </c>
     </row>
     <row r="4">
@@ -14778,7 +14778,7 @@
         <v>100</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>1.0549</v>
+        <v>0.4922</v>
       </c>
     </row>
     <row r="5">
@@ -14821,7 +14821,7 @@
         <v>100</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.7059</v>
+        <v>0.1106</v>
       </c>
     </row>
     <row r="6">
@@ -14864,7 +14864,7 @@
         <v>100</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>4.0509</v>
+        <v>1.598</v>
       </c>
     </row>
     <row r="7">
@@ -14907,7 +14907,7 @@
         <v>100</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>5.7203</v>
+        <v>1.7024</v>
       </c>
     </row>
     <row r="8">
@@ -14950,7 +14950,7 @@
         <v>100</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>6.5066</v>
+        <v>1.6724</v>
       </c>
     </row>
     <row r="9">
@@ -14993,7 +14993,7 @@
         <v>100</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0.6393</v>
+        <v>0.0303</v>
       </c>
     </row>
     <row r="10">
@@ -15036,7 +15036,7 @@
         <v>100</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.7682</v>
+        <v>0.0346</v>
       </c>
     </row>
     <row r="11">
@@ -15079,7 +15079,7 @@
         <v>100</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.9045</v>
+        <v>0.277</v>
       </c>
     </row>
     <row r="12">
@@ -15122,7 +15122,7 @@
         <v>100</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>1.3425</v>
+        <v>0.724</v>
       </c>
     </row>
     <row r="13">
@@ -15165,7 +15165,7 @@
         <v>100</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>1.0841</v>
+        <v>0.047</v>
       </c>
     </row>
     <row r="14">
@@ -15208,7 +15208,7 @@
         <v>100</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.7</v>
+        <v>0.0023</v>
       </c>
     </row>
     <row r="15">
@@ -15251,7 +15251,7 @@
         <v>100</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>1.4994</v>
+        <v>0.08110000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -15294,7 +15294,7 @@
         <v>100</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>1.5027</v>
+        <v>0.06850000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -15337,7 +15337,7 @@
         <v>100</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0.5279</v>
+        <v>0.0244</v>
       </c>
     </row>
     <row r="18">
@@ -15380,7 +15380,7 @@
         <v>100</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0.8023</v>
+        <v>0.0305</v>
       </c>
     </row>
     <row r="19">
@@ -15423,7 +15423,7 @@
         <v>100</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>1.0957</v>
+        <v>0.0427</v>
       </c>
     </row>
     <row r="20">
@@ -15466,7 +15466,7 @@
         <v>100</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1.4675</v>
+        <v>0.0641</v>
       </c>
     </row>
     <row r="21">
@@ -15509,7 +15509,7 @@
         <v>100</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>1.0067</v>
+        <v>0.0548</v>
       </c>
     </row>
     <row r="22">
@@ -15552,7 +15552,7 @@
         <v>100</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>1.1968</v>
+        <v>0.0497</v>
       </c>
     </row>
     <row r="23">
@@ -15595,7 +15595,7 @@
         <v>100</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>1.106</v>
+        <v>0.0399</v>
       </c>
     </row>
     <row r="24">
@@ -15638,7 +15638,7 @@
         <v>100</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0</v>
+        <v>0.0313</v>
       </c>
     </row>
     <row r="25">
@@ -15681,7 +15681,7 @@
         <v>100</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0.8504</v>
+        <v>0.043</v>
       </c>
     </row>
     <row r="26">
@@ -15724,7 +15724,7 @@
         <v>100</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>0.4797</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -15767,7 +15767,7 @@
         <v>100</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0.8186</v>
+        <v>0.0387</v>
       </c>
     </row>
     <row r="28">
@@ -15810,7 +15810,7 @@
         <v>100</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>1.0342</v>
+        <v>0.0601</v>
       </c>
     </row>
     <row r="29">
@@ -15853,7 +15853,7 @@
         <v>100</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>1.0473</v>
+        <v>0.0432</v>
       </c>
     </row>
     <row r="30">
@@ -15896,7 +15896,7 @@
         <v>100</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0.9177999999999999</v>
+        <v>0.0386</v>
       </c>
     </row>
     <row r="31">
@@ -15939,7 +15939,7 @@
         <v>100</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0.9507</v>
+        <v>0.0463</v>
       </c>
     </row>
     <row r="32">
@@ -15982,7 +15982,7 @@
         <v>100</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0.8407</v>
+        <v>0.0358</v>
       </c>
     </row>
     <row r="33">
@@ -16025,7 +16025,7 @@
         <v>100</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>0.7994</v>
+        <v>0.0409</v>
       </c>
     </row>
     <row r="34">
@@ -16068,7 +16068,7 @@
         <v>100</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0.7863</v>
+        <v>0.0374</v>
       </c>
     </row>
     <row r="35">
@@ -16111,7 +16111,7 @@
         <v>100</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0.9322</v>
+        <v>0.039</v>
       </c>
     </row>
     <row r="36">
@@ -16154,7 +16154,7 @@
         <v>100</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0.7668</v>
+        <v>0.0366</v>
       </c>
     </row>
     <row r="37">
@@ -16197,7 +16197,7 @@
         <v>100</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>0.7635</v>
+        <v>0.027</v>
       </c>
     </row>
     <row r="38">
@@ -16240,7 +16240,7 @@
         <v>100</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0.9029</v>
+        <v>0.0361</v>
       </c>
     </row>
     <row r="39">
@@ -16283,7 +16283,7 @@
         <v>100</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0.7647</v>
+        <v>0.0381</v>
       </c>
     </row>
     <row r="40">
@@ -16326,7 +16326,7 @@
         <v>100</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0.8577</v>
+        <v>0.0372</v>
       </c>
     </row>
     <row r="41">
@@ -16369,7 +16369,7 @@
         <v>100</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>1.0279</v>
+        <v>0.0386</v>
       </c>
     </row>
     <row r="42">
@@ -16412,7 +16412,7 @@
         <v>100</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0.8016</v>
+        <v>0.0331</v>
       </c>
     </row>
     <row r="43">
@@ -16455,7 +16455,7 @@
         <v>100</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0.7861</v>
+        <v>0.0371</v>
       </c>
     </row>
     <row r="44">
@@ -16498,7 +16498,7 @@
         <v>100</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.7359</v>
+        <v>0.0293</v>
       </c>
     </row>
     <row r="45">
@@ -16541,7 +16541,7 @@
         <v>100</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>0.736</v>
+        <v>0.0371</v>
       </c>
     </row>
     <row r="46">
@@ -16584,7 +16584,7 @@
         <v>100</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>0.8363</v>
+        <v>0.0413</v>
       </c>
     </row>
     <row r="47">
@@ -16627,7 +16627,7 @@
         <v>100</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.8976</v>
+        <v>0.0358</v>
       </c>
     </row>
     <row r="48">
@@ -16670,7 +16670,7 @@
         <v>100</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>1.0085</v>
+        <v>0.0364</v>
       </c>
     </row>
     <row r="49">
@@ -16713,7 +16713,7 @@
         <v>100</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>0.7968</v>
+        <v>0.0331</v>
       </c>
     </row>
     <row r="50">
@@ -16756,7 +16756,7 @@
         <v>100</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>0.6751</v>
+        <v>0.0382</v>
       </c>
     </row>
     <row r="51">
@@ -16799,7 +16799,7 @@
         <v>100</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>0.921</v>
+        <v>0.0345</v>
       </c>
     </row>
     <row r="52">
@@ -16842,7 +16842,7 @@
         <v>100</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.7968</v>
+        <v>0.0384</v>
       </c>
     </row>
     <row r="53">
@@ -16885,7 +16885,7 @@
         <v>100</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.9216</v>
+        <v>0.0441</v>
       </c>
     </row>
     <row r="54">
@@ -16928,7 +16928,7 @@
         <v>100</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.9298999999999999</v>
+        <v>0.038</v>
       </c>
     </row>
     <row r="55">
@@ -17014,7 +17014,7 @@
         <v>100</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0.6892</v>
+        <v>0.0387</v>
       </c>
     </row>
     <row r="57">
@@ -17057,7 +17057,7 @@
         <v>100</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.0366</v>
       </c>
     </row>
     <row r="58">
@@ -17100,7 +17100,7 @@
         <v>100</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.843</v>
+        <v>0.0311</v>
       </c>
     </row>
     <row r="59">
@@ -17143,7 +17143,7 @@
         <v>100</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.7106</v>
+        <v>0.0299</v>
       </c>
     </row>
     <row r="60">
@@ -17186,7 +17186,7 @@
         <v>100</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.9939</v>
+        <v>0.0404</v>
       </c>
     </row>
     <row r="61">
@@ -17229,7 +17229,7 @@
         <v>100</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>0.7329</v>
+        <v>0.0217</v>
       </c>
     </row>
     <row r="62">
@@ -17272,7 +17272,7 @@
         <v>100</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>0.8078</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="63">
@@ -17315,7 +17315,7 @@
         <v>100</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>0.8245</v>
+        <v>0.0361</v>
       </c>
     </row>
     <row r="64">
@@ -17358,7 +17358,7 @@
         <v>32.3</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>1.2721</v>
+        <v>0.06900000000000001</v>
       </c>
     </row>
     <row r="65">
@@ -17401,7 +17401,7 @@
         <v>48.4</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>0.6273</v>
+        <v>0.0342</v>
       </c>
     </row>
     <row r="66">
@@ -17444,7 +17444,7 @@
         <v>19.4</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>0.8405</v>
+        <v>0.037</v>
       </c>
     </row>
     <row r="67">
@@ -17487,7 +17487,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>0.8945</v>
+        <v>0.0378</v>
       </c>
     </row>
     <row r="68">
@@ -17530,7 +17530,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0.9424</v>
+        <v>0.0489</v>
       </c>
     </row>
     <row r="69">
@@ -17573,7 +17573,7 @@
         <v>67.7</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>1.0223</v>
+        <v>0.0375</v>
       </c>
     </row>
     <row r="70">
@@ -17616,7 +17616,7 @@
         <v>100</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>0.8672</v>
+        <v>0.0399</v>
       </c>
     </row>
     <row r="71">
@@ -17659,7 +17659,7 @@
         <v>100</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>0.825</v>
+        <v>0.0329</v>
       </c>
     </row>
     <row r="72">
@@ -17702,7 +17702,7 @@
         <v>100</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>0.8192</v>
+        <v>0.0431</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update NBA features + predictions: 2026-09-29 20:42
</commit_message>
<xml_diff>
--- a/nba-backend/data_delivery/nba_feature_workbook_20260929.xlsx
+++ b/nba-backend/data_delivery/nba_feature_workbook_20260929.xlsx
@@ -9356,7 +9356,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>91.0172</v>
+        <v>90.3948</v>
       </c>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
@@ -9369,7 +9369,7 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>1.7024</v>
+        <v>1.7196</v>
       </c>
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="n"/>
@@ -9382,7 +9382,7 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>1.6724</v>
+        <v>1.7041</v>
       </c>
       <c r="C19" s="2" t="n"/>
       <c r="D19" s="2" t="n"/>
@@ -9395,7 +9395,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>1.598</v>
+        <v>1.6098</v>
       </c>
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n"/>
@@ -9408,7 +9408,7 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>0.724</v>
+        <v>0.5954</v>
       </c>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
@@ -9421,7 +9421,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>0.4922</v>
+        <v>0.4889</v>
       </c>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n"/>
@@ -9430,11 +9430,11 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ewm_turnover_margin_diff</t>
+          <t>event_shooting_fouls_diff</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>0.277</v>
+        <v>0.3866</v>
       </c>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n"/>
@@ -9443,11 +9443,11 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>back_to_back_diff</t>
+          <t>ewm_turnover_margin_diff</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>0.1106</v>
+        <v>0.2503</v>
       </c>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
@@ -9456,11 +9456,11 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>elo_home</t>
+          <t>back_to_back_diff</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>0.08110000000000001</v>
+        <v>0.1119</v>
       </c>
       <c r="C25" s="2" t="n"/>
       <c r="D25" s="2" t="n"/>
@@ -9469,11 +9469,11 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>pl_ts_c_away</t>
+          <t>elo_home</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.0885</v>
       </c>
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="n"/>
@@ -9592,7 +9592,7 @@
         <v>100</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>91.0172</v>
+        <v>90.3948</v>
       </c>
     </row>
     <row r="3">
@@ -9635,7 +9635,7 @@
         <v>100</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0.0413</v>
+        <v>0.0483</v>
       </c>
     </row>
     <row r="4">
@@ -9678,7 +9678,7 @@
         <v>100</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.4922</v>
+        <v>0.4889</v>
       </c>
     </row>
     <row r="5">
@@ -9721,7 +9721,7 @@
         <v>100</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.1106</v>
+        <v>0.1119</v>
       </c>
     </row>
     <row r="6">
@@ -9764,7 +9764,7 @@
         <v>100</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1.598</v>
+        <v>1.6098</v>
       </c>
     </row>
     <row r="7">
@@ -9807,7 +9807,7 @@
         <v>100</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>1.7024</v>
+        <v>1.7196</v>
       </c>
     </row>
     <row r="8">
@@ -9850,7 +9850,7 @@
         <v>100</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>1.6724</v>
+        <v>1.7041</v>
       </c>
     </row>
     <row r="9">
@@ -9893,7 +9893,7 @@
         <v>100</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0.0303</v>
+        <v>0.0402</v>
       </c>
     </row>
     <row r="10">
@@ -9936,7 +9936,7 @@
         <v>100</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.0346</v>
+        <v>0.0419</v>
       </c>
     </row>
     <row r="11">
@@ -9979,7 +9979,7 @@
         <v>100</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.277</v>
+        <v>0.2503</v>
       </c>
     </row>
     <row r="12">
@@ -10022,7 +10022,7 @@
         <v>100</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0.724</v>
+        <v>0.5954</v>
       </c>
     </row>
     <row r="13">
@@ -10065,7 +10065,7 @@
         <v>100</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0.047</v>
+        <v>0.0483</v>
       </c>
     </row>
     <row r="14">
@@ -10108,7 +10108,7 @@
         <v>100</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0019</v>
       </c>
     </row>
     <row r="15">
@@ -10151,7 +10151,7 @@
         <v>100</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0.08110000000000001</v>
+        <v>0.0885</v>
       </c>
     </row>
     <row r="16">
@@ -10194,7 +10194,7 @@
         <v>100</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0.06850000000000001</v>
+        <v>0.0858</v>
       </c>
     </row>
     <row r="17">
@@ -10237,7 +10237,7 @@
         <v>100</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0.0244</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -10280,7 +10280,7 @@
         <v>100</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0.0305</v>
+        <v>0.0478</v>
       </c>
     </row>
     <row r="19">
@@ -10323,7 +10323,7 @@
         <v>100</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>0.0427</v>
+        <v>0.0519</v>
       </c>
     </row>
     <row r="20">
@@ -10366,7 +10366,7 @@
         <v>100</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0.0641</v>
+        <v>0.0726</v>
       </c>
     </row>
     <row r="21">
@@ -10409,7 +10409,7 @@
         <v>100</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>0.0548</v>
+        <v>0.07530000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -10452,7 +10452,7 @@
         <v>100</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>0.0497</v>
+        <v>0.0584</v>
       </c>
     </row>
     <row r="23">
@@ -10495,7 +10495,7 @@
         <v>100</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>0.0399</v>
+        <v>0.0557</v>
       </c>
     </row>
     <row r="24">
@@ -10538,7 +10538,7 @@
         <v>100</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0.0313</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -10581,7 +10581,7 @@
         <v>100</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0.043</v>
+        <v>0.0622</v>
       </c>
     </row>
     <row r="26">
@@ -10667,7 +10667,7 @@
         <v>100</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0.0387</v>
+        <v>0.0434</v>
       </c>
     </row>
     <row r="28">
@@ -10710,7 +10710,7 @@
         <v>100</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0.0601</v>
+        <v>0.0703</v>
       </c>
     </row>
     <row r="29">
@@ -10753,7 +10753,7 @@
         <v>100</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0.0432</v>
+        <v>0.0405</v>
       </c>
     </row>
     <row r="30">
@@ -10796,7 +10796,7 @@
         <v>100</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0.0386</v>
+        <v>0.0323</v>
       </c>
     </row>
     <row r="31">
@@ -10839,7 +10839,7 @@
         <v>100</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0.0463</v>
+        <v>0.0514</v>
       </c>
     </row>
     <row r="32">
@@ -10882,7 +10882,7 @@
         <v>100</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0.0358</v>
+        <v>0.0466</v>
       </c>
     </row>
     <row r="33">
@@ -10925,7 +10925,7 @@
         <v>100</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>0.0409</v>
+        <v>0.0434</v>
       </c>
     </row>
     <row r="34">
@@ -10968,7 +10968,7 @@
         <v>100</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0.0374</v>
+        <v>0.039</v>
       </c>
     </row>
     <row r="35">
@@ -11011,7 +11011,7 @@
         <v>100</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0.039</v>
+        <v>0.0488</v>
       </c>
     </row>
     <row r="36">
@@ -11054,7 +11054,7 @@
         <v>100</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0.0366</v>
+        <v>0.0439</v>
       </c>
     </row>
     <row r="37">
@@ -11097,7 +11097,7 @@
         <v>100</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>0.027</v>
+        <v>0.0383</v>
       </c>
     </row>
     <row r="38">
@@ -11140,7 +11140,7 @@
         <v>100</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0.0361</v>
+        <v>0.0411</v>
       </c>
     </row>
     <row r="39">
@@ -11183,7 +11183,7 @@
         <v>100</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0.0381</v>
+        <v>0.0403</v>
       </c>
     </row>
     <row r="40">
@@ -11226,7 +11226,7 @@
         <v>100</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0.0372</v>
+        <v>0.0415</v>
       </c>
     </row>
     <row r="41">
@@ -11269,7 +11269,7 @@
         <v>100</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>0.0386</v>
+        <v>0.0541</v>
       </c>
     </row>
     <row r="42">
@@ -11312,7 +11312,7 @@
         <v>100</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0.0331</v>
+        <v>0.0485</v>
       </c>
     </row>
     <row r="43">
@@ -11355,7 +11355,7 @@
         <v>100</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0.0371</v>
+        <v>0.054</v>
       </c>
     </row>
     <row r="44">
@@ -11398,7 +11398,7 @@
         <v>100</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.0293</v>
+        <v>0.047</v>
       </c>
     </row>
     <row r="45">
@@ -11441,7 +11441,7 @@
         <v>100</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>0.0371</v>
+        <v>0.0446</v>
       </c>
     </row>
     <row r="46">
@@ -11484,7 +11484,7 @@
         <v>100</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>0.0413</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -11527,7 +11527,7 @@
         <v>100</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.0358</v>
+        <v>0.0375</v>
       </c>
     </row>
     <row r="48">
@@ -11570,7 +11570,7 @@
         <v>100</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.0364</v>
+        <v>0.0376</v>
       </c>
     </row>
     <row r="49">
@@ -11613,7 +11613,7 @@
         <v>100</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>0.0331</v>
+        <v>0.0521</v>
       </c>
     </row>
     <row r="50">
@@ -11656,7 +11656,7 @@
         <v>100</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>0.0382</v>
+        <v>0.0377</v>
       </c>
     </row>
     <row r="51">
@@ -11742,7 +11742,7 @@
         <v>100</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.0384</v>
+        <v>0.0559</v>
       </c>
     </row>
     <row r="53">
@@ -11785,7 +11785,7 @@
         <v>100</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.0441</v>
+        <v>0.0448</v>
       </c>
     </row>
     <row r="54">
@@ -11828,7 +11828,7 @@
         <v>100</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.038</v>
+        <v>0.0412</v>
       </c>
     </row>
     <row r="55">
@@ -11914,7 +11914,7 @@
         <v>100</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0.0387</v>
+        <v>0.0446</v>
       </c>
     </row>
     <row r="57">
@@ -11957,7 +11957,7 @@
         <v>100</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.0366</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="58">
@@ -12000,7 +12000,7 @@
         <v>100</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.0311</v>
+        <v>0.0384</v>
       </c>
     </row>
     <row r="59">
@@ -12043,7 +12043,7 @@
         <v>100</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.0299</v>
+        <v>0.0365</v>
       </c>
     </row>
     <row r="60">
@@ -12086,7 +12086,7 @@
         <v>100</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.0404</v>
+        <v>0.0645</v>
       </c>
     </row>
     <row r="61">
@@ -12129,7 +12129,7 @@
         <v>100</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>0.0217</v>
+        <v>0.0436</v>
       </c>
     </row>
     <row r="62">
@@ -12172,7 +12172,7 @@
         <v>100</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>0.036</v>
+        <v>0.3866</v>
       </c>
     </row>
     <row r="63">
@@ -12215,7 +12215,7 @@
         <v>100</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>0.0361</v>
+        <v>0.0423</v>
       </c>
     </row>
     <row r="64">
@@ -12258,7 +12258,7 @@
         <v>32.3</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.064</v>
       </c>
     </row>
     <row r="65">
@@ -12301,7 +12301,7 @@
         <v>48.4</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>0.0342</v>
+        <v>0.0445</v>
       </c>
     </row>
     <row r="66">
@@ -12344,7 +12344,7 @@
         <v>19.4</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>0.037</v>
+        <v>0.0399</v>
       </c>
     </row>
     <row r="67">
@@ -12387,7 +12387,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>0.0378</v>
+        <v>0.0447</v>
       </c>
     </row>
     <row r="68">
@@ -12430,7 +12430,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0.0489</v>
+        <v>0.06320000000000001</v>
       </c>
     </row>
     <row r="69">
@@ -12473,7 +12473,7 @@
         <v>67.7</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>0.0375</v>
+        <v>0.0502</v>
       </c>
     </row>
     <row r="70">
@@ -12516,7 +12516,7 @@
         <v>100</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>0.0399</v>
+        <v>0.0494</v>
       </c>
     </row>
     <row r="71">
@@ -12559,7 +12559,7 @@
         <v>100</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>0.0329</v>
+        <v>0.0397</v>
       </c>
     </row>
     <row r="72">
@@ -12602,7 +12602,7 @@
         <v>100</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>0.0431</v>
+        <v>0.0525</v>
       </c>
     </row>
     <row r="73">
@@ -14692,7 +14692,7 @@
         <v>100</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>91.0172</v>
+        <v>90.3948</v>
       </c>
     </row>
     <row r="3">
@@ -14735,7 +14735,7 @@
         <v>100</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0.0413</v>
+        <v>0.0483</v>
       </c>
     </row>
     <row r="4">
@@ -14778,7 +14778,7 @@
         <v>100</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.4922</v>
+        <v>0.4889</v>
       </c>
     </row>
     <row r="5">
@@ -14821,7 +14821,7 @@
         <v>100</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.1106</v>
+        <v>0.1119</v>
       </c>
     </row>
     <row r="6">
@@ -14864,7 +14864,7 @@
         <v>100</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1.598</v>
+        <v>1.6098</v>
       </c>
     </row>
     <row r="7">
@@ -14907,7 +14907,7 @@
         <v>100</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>1.7024</v>
+        <v>1.7196</v>
       </c>
     </row>
     <row r="8">
@@ -14950,7 +14950,7 @@
         <v>100</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>1.6724</v>
+        <v>1.7041</v>
       </c>
     </row>
     <row r="9">
@@ -14993,7 +14993,7 @@
         <v>100</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0.0303</v>
+        <v>0.0402</v>
       </c>
     </row>
     <row r="10">
@@ -15036,7 +15036,7 @@
         <v>100</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.0346</v>
+        <v>0.0419</v>
       </c>
     </row>
     <row r="11">
@@ -15079,7 +15079,7 @@
         <v>100</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.277</v>
+        <v>0.2503</v>
       </c>
     </row>
     <row r="12">
@@ -15122,7 +15122,7 @@
         <v>100</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0.724</v>
+        <v>0.5954</v>
       </c>
     </row>
     <row r="13">
@@ -15165,7 +15165,7 @@
         <v>100</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0.047</v>
+        <v>0.0483</v>
       </c>
     </row>
     <row r="14">
@@ -15208,7 +15208,7 @@
         <v>100</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0019</v>
       </c>
     </row>
     <row r="15">
@@ -15251,7 +15251,7 @@
         <v>100</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0.08110000000000001</v>
+        <v>0.0885</v>
       </c>
     </row>
     <row r="16">
@@ -15294,7 +15294,7 @@
         <v>100</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0.06850000000000001</v>
+        <v>0.0858</v>
       </c>
     </row>
     <row r="17">
@@ -15337,7 +15337,7 @@
         <v>100</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0.0244</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -15380,7 +15380,7 @@
         <v>100</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0.0305</v>
+        <v>0.0478</v>
       </c>
     </row>
     <row r="19">
@@ -15423,7 +15423,7 @@
         <v>100</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>0.0427</v>
+        <v>0.0519</v>
       </c>
     </row>
     <row r="20">
@@ -15466,7 +15466,7 @@
         <v>100</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0.0641</v>
+        <v>0.0726</v>
       </c>
     </row>
     <row r="21">
@@ -15509,7 +15509,7 @@
         <v>100</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>0.0548</v>
+        <v>0.07530000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -15552,7 +15552,7 @@
         <v>100</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>0.0497</v>
+        <v>0.0584</v>
       </c>
     </row>
     <row r="23">
@@ -15595,7 +15595,7 @@
         <v>100</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>0.0399</v>
+        <v>0.0557</v>
       </c>
     </row>
     <row r="24">
@@ -15638,7 +15638,7 @@
         <v>100</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0.0313</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -15681,7 +15681,7 @@
         <v>100</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0.043</v>
+        <v>0.0622</v>
       </c>
     </row>
     <row r="26">
@@ -15767,7 +15767,7 @@
         <v>100</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0.0387</v>
+        <v>0.0434</v>
       </c>
     </row>
     <row r="28">
@@ -15810,7 +15810,7 @@
         <v>100</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0.0601</v>
+        <v>0.0703</v>
       </c>
     </row>
     <row r="29">
@@ -15853,7 +15853,7 @@
         <v>100</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0.0432</v>
+        <v>0.0405</v>
       </c>
     </row>
     <row r="30">
@@ -15896,7 +15896,7 @@
         <v>100</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0.0386</v>
+        <v>0.0323</v>
       </c>
     </row>
     <row r="31">
@@ -15939,7 +15939,7 @@
         <v>100</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0.0463</v>
+        <v>0.0514</v>
       </c>
     </row>
     <row r="32">
@@ -15982,7 +15982,7 @@
         <v>100</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0.0358</v>
+        <v>0.0466</v>
       </c>
     </row>
     <row r="33">
@@ -16025,7 +16025,7 @@
         <v>100</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>0.0409</v>
+        <v>0.0434</v>
       </c>
     </row>
     <row r="34">
@@ -16068,7 +16068,7 @@
         <v>100</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0.0374</v>
+        <v>0.039</v>
       </c>
     </row>
     <row r="35">
@@ -16111,7 +16111,7 @@
         <v>100</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0.039</v>
+        <v>0.0488</v>
       </c>
     </row>
     <row r="36">
@@ -16154,7 +16154,7 @@
         <v>100</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0.0366</v>
+        <v>0.0439</v>
       </c>
     </row>
     <row r="37">
@@ -16197,7 +16197,7 @@
         <v>100</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>0.027</v>
+        <v>0.0383</v>
       </c>
     </row>
     <row r="38">
@@ -16240,7 +16240,7 @@
         <v>100</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0.0361</v>
+        <v>0.0411</v>
       </c>
     </row>
     <row r="39">
@@ -16283,7 +16283,7 @@
         <v>100</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0.0381</v>
+        <v>0.0403</v>
       </c>
     </row>
     <row r="40">
@@ -16326,7 +16326,7 @@
         <v>100</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0.0372</v>
+        <v>0.0415</v>
       </c>
     </row>
     <row r="41">
@@ -16369,7 +16369,7 @@
         <v>100</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>0.0386</v>
+        <v>0.0541</v>
       </c>
     </row>
     <row r="42">
@@ -16412,7 +16412,7 @@
         <v>100</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0.0331</v>
+        <v>0.0485</v>
       </c>
     </row>
     <row r="43">
@@ -16455,7 +16455,7 @@
         <v>100</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0.0371</v>
+        <v>0.054</v>
       </c>
     </row>
     <row r="44">
@@ -16498,7 +16498,7 @@
         <v>100</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.0293</v>
+        <v>0.047</v>
       </c>
     </row>
     <row r="45">
@@ -16541,7 +16541,7 @@
         <v>100</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>0.0371</v>
+        <v>0.0446</v>
       </c>
     </row>
     <row r="46">
@@ -16584,7 +16584,7 @@
         <v>100</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>0.0413</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -16627,7 +16627,7 @@
         <v>100</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.0358</v>
+        <v>0.0375</v>
       </c>
     </row>
     <row r="48">
@@ -16670,7 +16670,7 @@
         <v>100</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.0364</v>
+        <v>0.0376</v>
       </c>
     </row>
     <row r="49">
@@ -16713,7 +16713,7 @@
         <v>100</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>0.0331</v>
+        <v>0.0521</v>
       </c>
     </row>
     <row r="50">
@@ -16756,7 +16756,7 @@
         <v>100</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>0.0382</v>
+        <v>0.0377</v>
       </c>
     </row>
     <row r="51">
@@ -16842,7 +16842,7 @@
         <v>100</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.0384</v>
+        <v>0.0559</v>
       </c>
     </row>
     <row r="53">
@@ -16885,7 +16885,7 @@
         <v>100</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.0441</v>
+        <v>0.0448</v>
       </c>
     </row>
     <row r="54">
@@ -16928,7 +16928,7 @@
         <v>100</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.038</v>
+        <v>0.0412</v>
       </c>
     </row>
     <row r="55">
@@ -17014,7 +17014,7 @@
         <v>100</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0.0387</v>
+        <v>0.0446</v>
       </c>
     </row>
     <row r="57">
@@ -17057,7 +17057,7 @@
         <v>100</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.0366</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="58">
@@ -17100,7 +17100,7 @@
         <v>100</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.0311</v>
+        <v>0.0384</v>
       </c>
     </row>
     <row r="59">
@@ -17143,7 +17143,7 @@
         <v>100</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.0299</v>
+        <v>0.0365</v>
       </c>
     </row>
     <row r="60">
@@ -17186,7 +17186,7 @@
         <v>100</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.0404</v>
+        <v>0.0645</v>
       </c>
     </row>
     <row r="61">
@@ -17229,7 +17229,7 @@
         <v>100</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>0.0217</v>
+        <v>0.0436</v>
       </c>
     </row>
     <row r="62">
@@ -17272,7 +17272,7 @@
         <v>100</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>0.036</v>
+        <v>0.3866</v>
       </c>
     </row>
     <row r="63">
@@ -17315,7 +17315,7 @@
         <v>100</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>0.0361</v>
+        <v>0.0423</v>
       </c>
     </row>
     <row r="64">
@@ -17358,7 +17358,7 @@
         <v>32.3</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.064</v>
       </c>
     </row>
     <row r="65">
@@ -17401,7 +17401,7 @@
         <v>48.4</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>0.0342</v>
+        <v>0.0445</v>
       </c>
     </row>
     <row r="66">
@@ -17444,7 +17444,7 @@
         <v>19.4</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>0.037</v>
+        <v>0.0399</v>
       </c>
     </row>
     <row r="67">
@@ -17487,7 +17487,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>0.0378</v>
+        <v>0.0447</v>
       </c>
     </row>
     <row r="68">
@@ -17530,7 +17530,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0.0489</v>
+        <v>0.06320000000000001</v>
       </c>
     </row>
     <row r="69">
@@ -17573,7 +17573,7 @@
         <v>67.7</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>0.0375</v>
+        <v>0.0502</v>
       </c>
     </row>
     <row r="70">
@@ -17616,7 +17616,7 @@
         <v>100</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>0.0399</v>
+        <v>0.0494</v>
       </c>
     </row>
     <row r="71">
@@ -17659,7 +17659,7 @@
         <v>100</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>0.0329</v>
+        <v>0.0397</v>
       </c>
     </row>
     <row r="72">
@@ -17702,7 +17702,7 @@
         <v>100</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>0.0431</v>
+        <v>0.0525</v>
       </c>
     </row>
   </sheetData>

</xml_diff>